<commit_message>
& - 86196888 от 18.02.2026 https://meshok.net/ - 86643117 от 04.03.2026 https://meshok.net/ - 26627 от 03.02.2026 https://2eurostore.ru/ - 26670 от 04.02.2026 https://2eurostore.ru/
</commit_message>
<xml_diff>
--- a/Collections/EURO/Estonia/#EURO#Estonia#Regular#[2011-present]#circulation_quality.xlsx
+++ b/Collections/EURO/Estonia/#EURO#Estonia#Regular#[2011-present]#circulation_quality.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lord_Alexator\Documents\CoinCollection\Collections\EURO\Estonia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14DB2512-1D2E-47BB-B517-25F65E995078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92194D99-1877-4883-9C62-9FB4F6C1B75C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1cent" sheetId="4" r:id="rId1"/>
@@ -1558,447 +1558,7 @@
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="142">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9BE5FF"/>
-          <bgColor rgb="FF9BE5FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="139">
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2007,6 +1567,422 @@
     </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -2711,9 +2687,9 @@
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="№" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Link" dataDxfId="56" dataCellStyle="Гиперссылка"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description (single table, table set, mintage, prices):" dataDxfId="55"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="№" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Link" dataDxfId="1" dataCellStyle="Гиперссылка"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description (single table, table set, mintage, prices):" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="1" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -3787,12 +3763,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3:K11">
-    <cfRule type="containsText" dxfId="141" priority="73" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="138" priority="73" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L3:L11">
-    <cfRule type="containsText" dxfId="140" priority="49" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="137" priority="49" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="50">
@@ -3807,7 +3783,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M3:M11">
-    <cfRule type="containsText" dxfId="139" priority="47" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="136" priority="47" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(M3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="48">
@@ -3822,7 +3798,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N3:N11">
-    <cfRule type="containsText" dxfId="138" priority="45" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="135" priority="45" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(N3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="46">
@@ -3837,7 +3813,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L12:L15">
-    <cfRule type="containsText" dxfId="137" priority="33" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="134" priority="33" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="34">
@@ -3852,7 +3828,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N12:N15">
-    <cfRule type="containsText" dxfId="136" priority="37" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="133" priority="37" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(N12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="38">
@@ -3867,7 +3843,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M12:M15">
-    <cfRule type="containsText" dxfId="135" priority="31" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="132" priority="31" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(M12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="32">
@@ -3894,12 +3870,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12:K15">
-    <cfRule type="containsText" dxfId="134" priority="35" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="131" priority="35" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J13 J15">
-    <cfRule type="containsText" dxfId="133" priority="29" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="130" priority="29" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="30">
@@ -3926,12 +3902,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J14">
-    <cfRule type="containsText" dxfId="132" priority="21" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="129" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L16">
-    <cfRule type="containsText" dxfId="54" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="128" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -3946,7 +3922,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N16">
-    <cfRule type="containsText" dxfId="53" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="127" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(N16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="20">
@@ -3961,7 +3937,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M16">
-    <cfRule type="containsText" dxfId="52" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="126" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(M16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -3988,12 +3964,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K16">
-    <cfRule type="containsText" dxfId="51" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="125" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="containsText" dxfId="50" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="124" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -4008,7 +3984,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L17">
-    <cfRule type="containsText" dxfId="49" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="123" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -4023,7 +3999,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N17">
-    <cfRule type="containsText" dxfId="48" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="122" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(N17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -4038,7 +4014,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M17">
-    <cfRule type="containsText" dxfId="47" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="121" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(M17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -4065,12 +4041,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K17">
-    <cfRule type="containsText" dxfId="46" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="120" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="containsText" dxfId="45" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="119" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -4361,7 +4337,7 @@
         <v>0</v>
       </c>
       <c r="L7" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M7" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4797,12 +4773,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J11">
-    <cfRule type="containsText" dxfId="131" priority="65" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="118" priority="65" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L3:L11">
-    <cfRule type="containsText" dxfId="130" priority="59" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="117" priority="59" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="60">
@@ -4829,12 +4805,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J12">
-    <cfRule type="containsText" dxfId="129" priority="49" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="116" priority="49" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L12">
-    <cfRule type="containsText" dxfId="128" priority="47" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="115" priority="47" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="48">
@@ -4861,12 +4837,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J13">
-    <cfRule type="containsText" dxfId="127" priority="45" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="114" priority="45" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L13">
-    <cfRule type="containsText" dxfId="126" priority="41" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="113" priority="41" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L13))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="42">
@@ -4881,7 +4857,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3:I12">
-    <cfRule type="containsText" dxfId="125" priority="39" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="112" priority="39" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="40">
@@ -4896,7 +4872,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I13">
-    <cfRule type="containsText" dxfId="124" priority="37" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="111" priority="37" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I13))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="38">
@@ -4923,12 +4899,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J14">
-    <cfRule type="containsText" dxfId="123" priority="31" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="110" priority="31" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I14">
-    <cfRule type="containsText" dxfId="122" priority="27" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="109" priority="27" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="28">
@@ -4955,12 +4931,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J15">
-    <cfRule type="containsText" dxfId="121" priority="25" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="108" priority="25" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L15">
-    <cfRule type="containsText" dxfId="120" priority="23" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="107" priority="23" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="24">
@@ -4975,7 +4951,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I15">
-    <cfRule type="containsText" dxfId="119" priority="21" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="106" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="22">
@@ -4990,7 +4966,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L14">
-    <cfRule type="containsText" dxfId="118" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="105" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="20">
@@ -5017,12 +4993,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="containsText" dxfId="41" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="104" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L16">
-    <cfRule type="containsText" dxfId="40" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="103" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -5037,7 +5013,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I16">
-    <cfRule type="containsText" dxfId="39" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="102" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -5064,12 +5040,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="containsText" dxfId="38" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="101" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(#REF!))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L17">
-    <cfRule type="containsText" dxfId="37" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="100" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(L17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -5084,7 +5060,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I17">
-    <cfRule type="containsText" dxfId="36" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="99" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -5707,7 +5683,7 @@
     <mergeCell ref="C1:D1"/>
   </mergeCells>
   <conditionalFormatting sqref="I3:I11 I13 I15">
-    <cfRule type="containsText" dxfId="117" priority="27" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="98" priority="27" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="28">
@@ -5722,7 +5698,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J11 J13 J15">
-    <cfRule type="containsText" dxfId="116" priority="25" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="97" priority="25" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="26">
@@ -5736,8 +5712,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14 I12">
-    <cfRule type="containsText" dxfId="115" priority="23" operator="containsText" text="*-">
+  <conditionalFormatting sqref="I12 I14">
+    <cfRule type="containsText" dxfId="96" priority="23" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="24">
@@ -5751,8 +5727,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J14 J12">
-    <cfRule type="containsText" dxfId="114" priority="21" operator="containsText" text="*-">
+  <conditionalFormatting sqref="J12 J14">
+    <cfRule type="containsText" dxfId="95" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="22">
@@ -5767,7 +5743,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15">
-    <cfRule type="containsText" dxfId="113" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="94" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -5782,7 +5758,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H12">
-    <cfRule type="containsText" dxfId="112" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="93" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="20">
@@ -5797,7 +5773,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="containsText" dxfId="111" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="92" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H13))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="18">
@@ -5812,7 +5788,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14">
-    <cfRule type="containsText" dxfId="110" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="91" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -5827,7 +5803,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I17">
-    <cfRule type="containsText" dxfId="35" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="90" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -5842,7 +5818,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="containsText" dxfId="34" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="89" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -5857,7 +5833,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I16">
-    <cfRule type="containsText" dxfId="33" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="88" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -5872,7 +5848,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="containsText" dxfId="32" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="87" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -5887,7 +5863,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="containsText" dxfId="31" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="86" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -5902,7 +5878,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H17">
-    <cfRule type="containsText" dxfId="30" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="85" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -6537,7 +6513,7 @@
     <mergeCell ref="E1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="I3:I11 I13">
-    <cfRule type="containsText" dxfId="109" priority="33" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="84" priority="33" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="34">
@@ -6552,7 +6528,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J11 J13">
-    <cfRule type="containsText" dxfId="108" priority="31" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="83" priority="31" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="32">
@@ -6567,7 +6543,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I12">
-    <cfRule type="containsText" dxfId="107" priority="29" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="82" priority="29" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="30">
@@ -6582,7 +6558,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J12">
-    <cfRule type="containsText" dxfId="106" priority="27" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="81" priority="27" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="28">
@@ -6597,7 +6573,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I14:I15">
-    <cfRule type="containsText" dxfId="105" priority="25" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="80" priority="25" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="26">
@@ -6612,7 +6588,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J14:J15">
-    <cfRule type="containsText" dxfId="104" priority="23" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="79" priority="23" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="24">
@@ -6627,7 +6603,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15">
-    <cfRule type="containsText" dxfId="103" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="78" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -6642,7 +6618,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H12">
-    <cfRule type="containsText" dxfId="102" priority="21" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="77" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="22">
@@ -6657,7 +6633,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="containsText" dxfId="101" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="76" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H13))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="20">
@@ -6672,7 +6648,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14">
-    <cfRule type="containsText" dxfId="100" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="75" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -6687,7 +6663,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I17">
-    <cfRule type="containsText" dxfId="29" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="74" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -6702,7 +6678,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="containsText" dxfId="28" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="73" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -6717,7 +6693,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I16">
-    <cfRule type="containsText" dxfId="27" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="72" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -6732,7 +6708,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="containsText" dxfId="26" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="71" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -6747,7 +6723,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="containsText" dxfId="25" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="70" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -6762,7 +6738,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H17">
-    <cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="69" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -7398,7 +7374,7 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="I3:I11">
-    <cfRule type="containsText" dxfId="99" priority="39" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="68" priority="39" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="40">
@@ -7413,7 +7389,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J11">
-    <cfRule type="containsText" dxfId="98" priority="37" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="67" priority="37" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="38">
@@ -7427,8 +7403,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14 I12">
-    <cfRule type="containsText" dxfId="97" priority="35" operator="containsText" text="*-">
+  <conditionalFormatting sqref="I12 I14">
+    <cfRule type="containsText" dxfId="66" priority="35" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="36">
@@ -7443,7 +7419,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J12">
-    <cfRule type="containsText" dxfId="96" priority="33" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="65" priority="33" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="34">
@@ -7457,8 +7433,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I15 I13">
-    <cfRule type="containsText" dxfId="95" priority="31" operator="containsText" text="*-">
+  <conditionalFormatting sqref="I13 I15">
+    <cfRule type="containsText" dxfId="64" priority="31" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I13))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="32">
@@ -7473,7 +7449,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J15">
-    <cfRule type="containsText" dxfId="94" priority="23" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="63" priority="23" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="24">
@@ -7488,7 +7464,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J13">
-    <cfRule type="containsText" dxfId="93" priority="27" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="62" priority="27" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J13))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="28">
@@ -7503,7 +7479,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J14">
-    <cfRule type="containsText" dxfId="92" priority="25" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="61" priority="25" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="26">
@@ -7518,7 +7494,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15">
-    <cfRule type="containsText" dxfId="91" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="60" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -7533,7 +7509,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H12">
-    <cfRule type="containsText" dxfId="90" priority="21" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="59" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="22">
@@ -7548,7 +7524,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14">
-    <cfRule type="containsText" dxfId="89" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="58" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="18">
@@ -7563,7 +7539,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="containsText" dxfId="88" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="57" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H13))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="20">
@@ -7578,7 +7554,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I17">
-    <cfRule type="containsText" dxfId="23" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="56" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -7593,7 +7569,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="containsText" dxfId="22" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="55" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -7608,7 +7584,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I16">
-    <cfRule type="containsText" dxfId="21" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="54" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -7623,7 +7599,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="containsText" dxfId="20" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="53" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -7638,7 +7614,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="containsText" dxfId="19" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="52" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -7653,7 +7629,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H17">
-    <cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="51" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -8288,7 +8264,7 @@
     <mergeCell ref="E1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="I3:I11">
-    <cfRule type="containsText" dxfId="87" priority="39" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="50" priority="39" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="40">
@@ -8303,7 +8279,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J11">
-    <cfRule type="containsText" dxfId="86" priority="37" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="49" priority="37" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="38">
@@ -8318,7 +8294,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I12">
-    <cfRule type="containsText" dxfId="85" priority="35" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="48" priority="35" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="36">
@@ -8333,7 +8309,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J12">
-    <cfRule type="containsText" dxfId="84" priority="33" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="47" priority="33" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="34">
@@ -8348,7 +8324,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15">
-    <cfRule type="containsText" dxfId="83" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="46" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -8363,7 +8339,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H12">
-    <cfRule type="containsText" dxfId="82" priority="31" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="45" priority="31" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="32">
@@ -8378,7 +8354,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14">
-    <cfRule type="containsText" dxfId="81" priority="15" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="44" priority="15" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="16">
@@ -8392,8 +8368,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I15 I13">
-    <cfRule type="containsText" dxfId="80" priority="25" operator="containsText" text="*-">
+  <conditionalFormatting sqref="I13 I15">
+    <cfRule type="containsText" dxfId="43" priority="25" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I13))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="26">
@@ -8407,8 +8383,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J15 J13">
-    <cfRule type="containsText" dxfId="79" priority="23" operator="containsText" text="*-">
+  <conditionalFormatting sqref="J13 J15">
+    <cfRule type="containsText" dxfId="42" priority="23" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J13))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="24">
@@ -8423,7 +8399,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I14">
-    <cfRule type="containsText" dxfId="78" priority="21" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="41" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="22">
@@ -8438,7 +8414,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J14">
-    <cfRule type="containsText" dxfId="77" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="40" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="20">
@@ -8453,7 +8429,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13">
-    <cfRule type="containsText" dxfId="76" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="39" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H13))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="18">
@@ -8468,7 +8444,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I17">
-    <cfRule type="containsText" dxfId="17" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="38" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -8483,7 +8459,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="containsText" dxfId="16" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="37" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -8498,7 +8474,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I16">
-    <cfRule type="containsText" dxfId="15" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="36" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -8513,7 +8489,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="containsText" dxfId="14" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="35" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -8528,7 +8504,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="containsText" dxfId="13" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="34" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -8543,7 +8519,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H17">
-    <cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -9178,7 +9154,7 @@
     <mergeCell ref="E1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="I3:I11 I13 I15">
-    <cfRule type="containsText" dxfId="75" priority="27" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="32" priority="27" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="28">
@@ -9193,7 +9169,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J11 J13 J15">
-    <cfRule type="containsText" dxfId="74" priority="25" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="31" priority="25" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="26">
@@ -9207,8 +9183,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14 I12">
-    <cfRule type="containsText" dxfId="73" priority="23" operator="containsText" text="*-">
+  <conditionalFormatting sqref="I12 I14">
+    <cfRule type="containsText" dxfId="30" priority="23" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="24">
@@ -9222,8 +9198,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J14 J12">
-    <cfRule type="containsText" dxfId="72" priority="21" operator="containsText" text="*-">
+  <conditionalFormatting sqref="J12 J14">
+    <cfRule type="containsText" dxfId="29" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="22">
@@ -9238,7 +9214,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H13">
-    <cfRule type="containsText" dxfId="71" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="28" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="20">
@@ -9253,7 +9229,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14">
-    <cfRule type="containsText" dxfId="70" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="27" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="18">
@@ -9268,7 +9244,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15">
-    <cfRule type="containsText" dxfId="69" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="26" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -9283,7 +9259,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I17">
-    <cfRule type="containsText" dxfId="11" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="25" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -9298,7 +9274,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="containsText" dxfId="10" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="24" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -9313,7 +9289,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I16">
-    <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="23" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -9328,7 +9304,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="containsText" dxfId="8" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="22" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -9343,7 +9319,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="21" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -9358,7 +9334,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H17">
-    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="20" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">
@@ -10005,7 +9981,7 @@
     <mergeCell ref="C1:D1"/>
   </mergeCells>
   <conditionalFormatting sqref="I3:I11">
-    <cfRule type="containsText" dxfId="68" priority="35" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="19" priority="35" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="36">
@@ -10020,7 +9996,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J11">
-    <cfRule type="containsText" dxfId="67" priority="33" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="18" priority="33" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="34">
@@ -10035,7 +10011,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I12:I13">
-    <cfRule type="containsText" dxfId="66" priority="31" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="17" priority="31" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="32">
@@ -10050,7 +10026,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J12:J13">
-    <cfRule type="containsText" dxfId="65" priority="29" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="16" priority="29" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J12))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="30">
@@ -10065,7 +10041,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H13">
-    <cfRule type="containsText" dxfId="64" priority="27" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="15" priority="27" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="28">
@@ -10080,7 +10056,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I14">
-    <cfRule type="containsText" dxfId="63" priority="25" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="14" priority="25" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="26">
@@ -10095,7 +10071,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J14">
-    <cfRule type="containsText" dxfId="62" priority="23" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="13" priority="23" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="24">
@@ -10110,7 +10086,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14">
-    <cfRule type="containsText" dxfId="61" priority="21" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="12" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H14))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="22">
@@ -10125,7 +10101,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I15">
-    <cfRule type="containsText" dxfId="60" priority="19" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="11" priority="19" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="20">
@@ -10140,7 +10116,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J15">
-    <cfRule type="containsText" dxfId="59" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="10" priority="17" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="18">
@@ -10155,7 +10131,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H15">
-    <cfRule type="containsText" dxfId="58" priority="13" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="9" priority="13" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H15))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="14">
@@ -10170,7 +10146,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I17">
-    <cfRule type="containsText" dxfId="5" priority="11" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="8" priority="11" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="12">
@@ -10185,7 +10161,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J17">
-    <cfRule type="containsText" dxfId="4" priority="9" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="7" priority="9" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="10">
@@ -10200,7 +10176,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I16">
-    <cfRule type="containsText" dxfId="3" priority="7" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(I16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="8">
@@ -10215,7 +10191,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(J16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="6">
@@ -10230,7 +10206,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H16">
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H16))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -10245,7 +10221,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H17">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H17))))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="2">

</xml_diff>